<commit_message>
feat: add sorting functionality to contract and quotation managers for improved data organization
</commit_message>
<xml_diff>
--- a/baogiaxlsx.xlsx
+++ b/baogiaxlsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\laravel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC6B236A-B3D8-41F2-84E1-BB7E303AC930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F23138AB-73D9-4BF4-B47A-E97D4DBDA9E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{97C2FBF2-6402-49C5-AE5B-D1F0DBD5D27E}"/>
+    <workbookView xWindow="43080" yWindow="2595" windowWidth="29040" windowHeight="15720" xr2:uid="{97C2FBF2-6402-49C5-AE5B-D1F0DBD5D27E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="60">
   <si>
     <t>STT</t>
   </si>
@@ -81,9 +79,6 @@
   </si>
   <si>
     <t>GIÁ TRỊ HĐ (chưa VAT)</t>
-  </si>
-  <si>
-    <t>26/12/2025</t>
   </si>
   <si>
     <t>Công ty TNHH Công nghiệp Siêu Phàm 
@@ -119,9 +114,6 @@
     <t>52.000.000 đ</t>
   </si>
   <si>
-    <t>23/12/2025</t>
-  </si>
-  <si>
     <t>CÔNG TY TNHH MTV DỆT KIM 
 ĐÔNG PHƯƠNG(VN)</t>
   </si>
@@ -145,9 +137,6 @@
     <t>0 đ</t>
   </si>
   <si>
-    <t>24/12/2025</t>
-  </si>
-  <si>
     <t>CÔNG TY CỔ PHẦN VIETSTAR MEIDEN</t>
   </si>
   <si>
@@ -162,9 +151,6 @@
   </si>
   <si>
     <t>Bạn Huynh Vy;</t>
-  </si>
-  <si>
-    <t>22/12/2025</t>
   </si>
   <si>
     <t>CÔNG TY CỔ PHẦN TÔN POMINA</t>
@@ -190,9 +176,6 @@
   </si>
   <si>
     <t>29.110.000 đ</t>
-  </si>
-  <si>
-    <t>24/1/2026</t>
   </si>
   <si>
     <t xml:space="preserve">CÔNG TY DỊCH VỤ SỬA CHỮA CÁC NHÀ MÁY ĐIỆN EVNGENCO3
@@ -342,9 +325,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -352,6 +332,9 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -804,49 +787,49 @@
       <c r="AA1" s="2"/>
       <c r="AB1" s="2"/>
     </row>
-    <row r="2" spans="1:28" ht="92.25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:28" ht="107.65" x14ac:dyDescent="0.45">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="10">
+        <v>49672</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
@@ -867,44 +850,44 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="10">
+        <v>49673</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="F3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>29</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="N3" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
@@ -920,49 +903,49 @@
       <c r="AA3" s="2"/>
       <c r="AB3" s="2"/>
     </row>
-    <row r="4" spans="1:28" ht="92.25" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:28" ht="107.65" x14ac:dyDescent="0.45">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="10">
+        <v>46022</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>38</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="K4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="N4" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
@@ -983,44 +966,44 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="10">
+        <v>46023</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>44</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
@@ -1041,44 +1024,44 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>48</v>
+        <v>56</v>
+      </c>
+      <c r="C6" s="10">
+        <v>46024</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L6" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>50</v>
-      </c>
       <c r="M6" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
@@ -1099,44 +1082,44 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="7">
-        <v>46174</v>
-      </c>
-      <c r="D7" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="10">
+        <v>46025</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="6"/>
+      <c r="I7" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="K7" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="M7" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="N7" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="6"/>
-      <c r="I7" s="9" t="s">
+      <c r="O7" s="7" t="s">
         <v>55</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="K7" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="L7" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="M7" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="N7" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="O7" s="8" t="s">
-        <v>60</v>
       </c>
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
@@ -1154,6 +1137,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>